<commit_message>
📊 Auto scan: 2026-10-26
</commit_message>
<xml_diff>
--- a/archive/2026-10-26/report.xlsx
+++ b/archive/2026-10-26/report.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -600,10 +600,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -652,7 +652,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>스토킹</t>
+          <t>cve-2026-111497</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -681,7 +681,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tre tucker</t>
+          <t>erin andrews</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -710,7 +710,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>天気</t>
+          <t>new york state police</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -739,7 +739,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>josh jacobs</t>
+          <t>필리핀</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -768,7 +768,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>lyon</t>
+          <t>넾다세일</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>chris sorensen</t>
+          <t>76ers score</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -826,7 +826,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>บาร์ซา พบ เรอัลมาดริด</t>
+          <t>zach lavine</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -855,7 +855,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>pistons vs 76ers</t>
+          <t>인플루언서</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -884,7 +884,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>天气</t>
+          <t>카드뉴스</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -913,7 +913,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>atlas - puebla</t>
+          <t>cedric coward</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -942,7 +942,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>resultados das eleições</t>
+          <t>빌 게이츠</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -971,7 +971,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>이시영</t>
+          <t>rashid shaheed</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1000,7 +1000,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lcs</t>
+          <t>john collins</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1029,7 +1029,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>atlético nacional - medellín</t>
+          <t>시내버스</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1058,7 +1058,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cisse packers</t>
+          <t>탈세</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1087,7 +1087,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>barca</t>
+          <t>mikal bridges</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1116,7 +1116,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>이다해</t>
+          <t>jaylen wells</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1145,7 +1145,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>loteria nacional</t>
+          <t>우리은행</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1174,7 +1174,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>손지창</t>
+          <t>엘에이 fc 대 la 갤럭시</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1203,7 +1203,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>david moulton</t>
+          <t>isaiah stewart</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1247,11 +1247,11 @@
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="23">
@@ -1282,7 +1282,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>체코 원전</t>
+          <t>필러</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1297,17 +1297,17 @@
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
-        <v>1.6</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>체코원전</t>
+          <t>체코 원전</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1322,17 +1322,17 @@
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="n">
-        <v>1.6</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>필러</t>
+          <t>체코원전</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1347,17 +1347,17 @@
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
-        <v>1.63</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AI 인프라</t>
+          <t>투바투</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1372,85 +1372,10 @@
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>투바투</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>naver</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>47</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="n">
-        <v>1.59</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2차전지</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>naver</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="n">
-        <v>46</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="n">
-        <v>1.55</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>이차전지</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>naver</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>45</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="n">
         <v>1.53</v>
       </c>
     </row>
@@ -12144,14 +12069,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
@@ -12232,12 +12157,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>065770</t>
+          <t>053800</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>안랩</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -12246,26 +12171,26 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>766</v>
+        <v>78400</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>[직접매칭]</t>
+          <t>사이버보안</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>58.6</v>
+        <v>61.4</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>⚪ 관찰</t>
+          <t>🟡 주목</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>60</v>
       </c>
       <c r="I2" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="J2" t="n">
         <v>25</v>
@@ -12275,41 +12200,41 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>lcs</t>
+          <t>cedric coward</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>[직접매칭] 종목명 'CS'이 트렌드 키워드와 매칭. 거래량 시그널 60점 (2주avg/4-8주avg = 4.26, 2주/2-4주 = 1.31). 트렌드 시그널 76점 — 매칭: lcs(google, 76점).</t>
+          <t>[테마: 사이버보안] 거래량 시그널 60점 (2주avg/4-8주avg = 3.99, 2주/2-4주 = 1.54). 트렌드 시그널 84점 — 매칭 키워드: cedric coward(google, 84점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 엔드포인트 보안</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>086520</t>
+          <t>006260</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>72700</v>
+        <v>216500</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2차전지/배터리</t>
+          <t>[직접매칭]</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>58.1</v>
+        <v>50.8</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -12317,54 +12242,54 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>49.2</v>
+        <v>48.9</v>
       </c>
       <c r="I3" t="n">
-        <v>45.5</v>
+        <v>68</v>
       </c>
       <c r="J3" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="K3" t="b">
         <v>0</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2차전지, 이차전지</t>
+          <t>jaylen wells</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>[테마: 2차전지/배터리] 거래량 시그널 49점 (2주avg/4-8주avg = 1.64, 2주/2-4주 = 1.08). 트렌드 시그널 46점 — 매칭 키워드: 2차전지(naver, 46점), 이차전지(naver, 45점). 동일 테마 동시통과 4종목(밀집도 100점). 종목 근거: 양극재 지주</t>
+          <t>[직접매칭] 종목명 'LS'이 트렌드 키워드와 매칭. 거래량 시그널 49점 (2주avg/4-8주avg = 1.63, 2주/2-4주 = 1.04). 트렌드 시그널 68점 — 매칭: jaylen wells(google, 68점).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>121600</t>
+          <t>352820</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>나노신소재</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>55800</v>
+        <v>176500</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2차전지/배터리</t>
+          <t>K-콘텐츠/엔터</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>57.9</v>
+        <v>47.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -12372,245 +12297,25 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>48.8</v>
+        <v>53.7</v>
       </c>
       <c r="I4" t="n">
-        <v>45.5</v>
+        <v>52.5</v>
       </c>
       <c r="J4" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="K4" t="b">
         <v>0</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2차전지, 이차전지</t>
+          <t>아이브, 투바투</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>[테마: 2차전지/배터리] 거래량 시그널 49점 (2주avg/4-8주avg = 1.63, 2주/2-4주 = 1.08). 트렌드 시그널 46점 — 매칭 키워드: 2차전지(naver, 46점), 이차전지(naver, 45점). 동일 테마 동시통과 4종목(밀집도 100점). 종목 근거: CNT 도전재</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>373220</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>LG에너지솔루션</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>383000</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2차전지/배터리</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>57.6</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>⚪ 관찰</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>48.2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="J5" t="n">
-        <v>100</v>
-      </c>
-      <c r="K5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2차전지, 이차전지</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>[테마: 2차전지/배터리] 거래량 시그널 48점 (2주avg/4-8주avg = 1.61, 2주/2-4주 = 1.40). 트렌드 시그널 46점 — 매칭 키워드: 2차전지(naver, 46점), 이차전지(naver, 45점). 동일 테마 동시통과 4종목(밀집도 100점). 종목 근거: 글로벌 2위 셀</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>247540</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>에코프로비엠</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>KOSDAQ</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>92800</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2차전지/배터리</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>55.5</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>⚪ 관찰</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="I6" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="J6" t="n">
-        <v>100</v>
-      </c>
-      <c r="K6" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2차전지, 이차전지</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>[테마: 2차전지/배터리] 거래량 시그널 43점 (2주avg/4-8주avg = 1.45, 2주/2-4주 = 1.06). 트렌드 시그널 46점 — 매칭 키워드: 2차전지(naver, 46점), 이차전지(naver, 45점). 동일 테마 동시통과 4종목(밀집도 100점). 종목 근거: 양극재</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>352820</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>하이브</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>176500</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>K-콘텐츠/엔터</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>⚪ 관찰</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="I7" t="n">
-        <v>53</v>
-      </c>
-      <c r="J7" t="n">
-        <v>25</v>
-      </c>
-      <c r="K7" t="b">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>아이브, 투바투</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>[테마: K-콘텐츠/엔터] 거래량 시그널 54점 (2주avg/4-8주avg = 1.79, 2주/2-4주 = 1.50). 트렌드 시그널 53점 — 매칭 키워드: 아이브(naver, 59점), 투바투(naver, 47점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: BTS·뉴진스</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>418550</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>제이앤티씨</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>KOSDAQ</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>4320</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>데이터센터/AI인프라</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="I8" t="n">
-        <v>47</v>
-      </c>
-      <c r="J8" t="n">
-        <v>25</v>
-      </c>
-      <c r="K8" t="b">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>AI 인프라</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>[테마: 데이터센터/AI인프라] 거래량 시그널 42점 (2주avg/4-8주avg = 1.41, 2주/2-4주 = 1.04). 트렌드 시그널 47점 — 매칭 키워드: AI 인프라(naver, 47점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 광커넥터</t>
+          <t>[테마: K-콘텐츠/엔터] 거래량 시그널 54점 (2주avg/4-8주avg = 1.79, 2주/2-4주 = 1.50). 트렌드 시그널 52점 — 매칭 키워드: 아이브(naver, 60점), 투바투(naver, 45점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: BTS·뉴진스</t>
         </is>
       </c>
     </row>

</xml_diff>